<commit_message>
Add wav2vec plugins and model description UI. Added evidence for report
Register and add three new Wav2Vec-based classifier plugins (Leinster vs Rest, Ulster/Leinster/Rest, Province 4-way) that load joblib artifacts and provide predict() outputs. Update plugin loader to register the new plugins and bump FastAPI app title to Prototype4. Frontend: add model description UI, wire description rendering into model selection and prediction flows, update map highlighting to consider model-specific label-to-region logic and normalized province names, and pass model IDs to map updates. Also update module imports/versioned script tags, adjust some CSS, and add FinalReport Gantt chart and chart/image evidence files while removing a few archived interim report documents.
</commit_message>
<xml_diff>
--- a/FinalReport/Evidence/speaker_counts.xlsx
+++ b/FinalReport/Evidence/speaker_counts.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cianan/Documents/College/GitHub/FYP/FinalReport/Evidence/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88D38EF0-04CF-F44A-B2F5-2E41A79445BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{173C4406-83B3-7D4D-98E7-498ED7D83572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="1340" windowWidth="38400" windowHeight="23520" xr2:uid="{33F6CCAC-11FD-904F-A4EA-8A34A3E80E40}"/>
+    <workbookView xWindow="2640" yWindow="3140" windowWidth="27240" windowHeight="16440" xr2:uid="{33F6CCAC-11FD-904F-A4EA-8A34A3E80E40}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="21">
   <si>
     <t>Task</t>
   </si>
@@ -96,6 +96,9 @@
   </si>
   <si>
     <t>Northern Ireland</t>
+  </si>
+  <si>
+    <t>Percent</t>
   </si>
 </sst>
 </file>
@@ -230,6 +233,23 @@
     <tableColumn id="1" xr3:uid="{EEE1CDC9-BBBC-8046-88C0-FBAFC67914CD}" name="Class"/>
     <tableColumn id="2" xr3:uid="{04D0D358-E0CE-1C4C-8DF1-A1534AF52550}" name="Samples"/>
     <tableColumn id="3" xr3:uid="{F6EEC234-BF20-0A40-9A45-39FC2F2A54C9}" name="Speakers"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{E81C0688-1F1F-084F-9FC2-26D728B9390A}" name="Table59" displayName="Table59" ref="AE3:AG8" totalsRowCount="1">
+  <autoFilter ref="AE3:AG7" xr:uid="{E81C0688-1F1F-084F-9FC2-26D728B9390A}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{D905DFA4-9DDA-7343-B791-BADA0404329E}" name="Class"/>
+    <tableColumn id="2" xr3:uid="{25CF7464-5C2F-1247-84B4-DF120D2EB9BF}" name="Samples" totalsRowFunction="custom">
+      <totalsRowFormula>SUM(Table59[Samples])</totalsRowFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{5217A91D-2A10-3F47-A4D1-C37E3155E17C}" name="Percent" totalsRowFunction="custom">
+      <calculatedColumnFormula>(Table59[[#This Row],[Samples]]/Table59[[#Totals],[Samples]])*100</calculatedColumnFormula>
+      <totalsRowFormula>SUM(Table59[Percent])</totalsRowFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -552,7 +572,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C479BD2-4988-B940-8B72-6465756E4216}">
-  <dimension ref="B2:AC8"/>
+  <dimension ref="B2:AG8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="24.33203125" customWidth="1"/>
@@ -561,7 +581,7 @@
     <col min="27" max="27" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:29" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:33" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -593,7 +613,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:29" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:33" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>9</v>
       </c>
@@ -660,8 +680,17 @@
       <c r="AC3" t="s">
         <v>3</v>
       </c>
+      <c r="AE3" t="s">
+        <v>10</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>2</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="4" spans="2:29" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:33" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>4</v>
       </c>
@@ -728,8 +757,18 @@
       <c r="AC4">
         <v>195</v>
       </c>
+      <c r="AE4" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF4">
+        <v>481</v>
+      </c>
+      <c r="AG4">
+        <f>(Table59[[#This Row],[Samples]]/Table59[[#Totals],[Samples]])*100</f>
+        <v>29.728059332509272</v>
+      </c>
     </row>
-    <row r="5" spans="2:29" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:33" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>5</v>
       </c>
@@ -796,8 +835,18 @@
       <c r="AC5">
         <v>11</v>
       </c>
+      <c r="AE5" t="s">
+        <v>13</v>
+      </c>
+      <c r="AF5">
+        <v>541</v>
+      </c>
+      <c r="AG5">
+        <f>(Table59[[#This Row],[Samples]]/Table59[[#Totals],[Samples]])*100</f>
+        <v>33.436341161928304</v>
+      </c>
     </row>
-    <row r="6" spans="2:29" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:33" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>7</v>
       </c>
@@ -837,8 +886,18 @@
       <c r="Y6">
         <v>32</v>
       </c>
+      <c r="AE6" t="s">
+        <v>16</v>
+      </c>
+      <c r="AF6">
+        <v>249</v>
+      </c>
+      <c r="AG6">
+        <f>(Table59[[#This Row],[Samples]]/Table59[[#Totals],[Samples]])*100</f>
+        <v>15.389369592089</v>
+      </c>
     </row>
-    <row r="7" spans="2:29" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:33" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>8</v>
       </c>
@@ -869,8 +928,18 @@
       <c r="Y7">
         <v>52</v>
       </c>
+      <c r="AE7" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF7">
+        <v>347</v>
+      </c>
+      <c r="AG7">
+        <f>(Table59[[#This Row],[Samples]]/Table59[[#Totals],[Samples]])*100</f>
+        <v>21.446229913473424</v>
+      </c>
     </row>
-    <row r="8" spans="2:29" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:33" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>6</v>
       </c>
@@ -882,11 +951,19 @@
       </c>
       <c r="E8">
         <v>212</v>
+      </c>
+      <c r="AF8">
+        <f>SUM(Table59[Samples])</f>
+        <v>1618</v>
+      </c>
+      <c r="AG8">
+        <f>SUM(Table59[Percent])</f>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="7">
+  <tableParts count="8">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
@@ -894,6 +971,7 @@
     <tablePart r:id="rId5"/>
     <tablePart r:id="rId6"/>
     <tablePart r:id="rId7"/>
+    <tablePart r:id="rId8"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>